<commit_message>
Se finaliza sprint 5 - /status
</commit_message>
<xml_diff>
--- a/docs/Sprints.xlsx
+++ b/docs/Sprints.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADOS\Documents\CatEater\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B857EA8-2C16-470A-994C-4440C12F7989}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8303F0D9-40C3-4A87-BF2F-EA6C8AC23A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="1575" windowWidth="20730" windowHeight="11040" xr2:uid="{B0A1328C-A2DF-43BD-A97C-AEC866E5EF49}"/>
   </bookViews>
@@ -688,7 +688,9 @@
       <c r="C8" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="4"/>
+      <c r="D8" s="4">
+        <v>46225</v>
+      </c>
     </row>
     <row r="9" spans="1:4" ht="45">
       <c r="A9" s="3" t="s">

</xml_diff>

<commit_message>
Adiciones del endpoint /config, el cual configura los steps del motor
</commit_message>
<xml_diff>
--- a/docs/Sprints.xlsx
+++ b/docs/Sprints.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADOS\Documents\CatEater\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8303F0D9-40C3-4A87-BF2F-EA6C8AC23A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31A4D603-DDBF-432D-95C1-BF4A982A0D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="1575" windowWidth="20730" windowHeight="11040" xr2:uid="{B0A1328C-A2DF-43BD-A97C-AEC866E5EF49}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
   <si>
     <t>Sprint</t>
   </si>
@@ -169,6 +169,24 @@
   </si>
   <si>
     <t>Sistema de Configuración</t>
+  </si>
+  <si>
+    <t>6.1</t>
+  </si>
+  <si>
+    <t>Motor configurable</t>
+  </si>
+  <si>
+    <t>6.2</t>
+  </si>
+  <si>
+    <t>6.3</t>
+  </si>
+  <si>
+    <t>Nuevo endpoint PUT /config</t>
+  </si>
+  <si>
+    <t>GET /config</t>
   </si>
 </sst>
 </file>
@@ -266,8 +284,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A61D0C2F-3863-49B5-9DBD-2A45D434E86B}" name="Tabla1" displayName="Tabla1" ref="A2:D13" totalsRowShown="0">
-  <autoFilter ref="A2:D13" xr:uid="{A61D0C2F-3863-49B5-9DBD-2A45D434E86B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A61D0C2F-3863-49B5-9DBD-2A45D434E86B}" name="Tabla1" displayName="Tabla1" ref="A2:D17" totalsRowShown="0">
+  <autoFilter ref="A2:D17" xr:uid="{A61D0C2F-3863-49B5-9DBD-2A45D434E86B}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{D3E4F5C6-AD58-47DC-B6D4-1B0C795F5FB6}" name="Columna1" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{1A70B391-4605-4E18-BEE1-E86883F9110B}" name="Columna2" dataDxfId="1"/>
@@ -575,7 +593,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AD8F467-8232-41EB-8FA5-FE5849A43A27}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -704,48 +722,84 @@
       </c>
       <c r="D9" s="4"/>
     </row>
-    <row r="10" spans="1:4" ht="30">
+    <row r="10" spans="1:4" ht="45">
       <c r="A10" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>28</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="3"/>
       <c r="D10" s="4"/>
     </row>
-    <row r="11" spans="1:4" ht="30">
+    <row r="11" spans="1:4" ht="45">
       <c r="A11" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>30</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="4"/>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="3"/>
+      <c r="D12" s="4"/>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="3"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="4"/>
+    </row>
+    <row r="14" spans="1:4" ht="30">
+      <c r="A14" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" s="4"/>
+    </row>
+    <row r="15" spans="1:4" ht="30">
+      <c r="A15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B16" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="30">
-      <c r="A13" s="3" t="s">
+    <row r="17" spans="1:3" ht="30">
+      <c r="A17" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B17" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C17" s="3" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Primeras configuraciones de el storage
</commit_message>
<xml_diff>
--- a/docs/Sprints.xlsx
+++ b/docs/Sprints.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADOS\Documents\CatEater\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31A4D603-DDBF-432D-95C1-BF4A982A0D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FC3ABB8-A4DC-47EB-86CC-0636496B2FF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="1575" windowWidth="20730" windowHeight="11040" xr2:uid="{B0A1328C-A2DF-43BD-A97C-AEC866E5EF49}"/>
   </bookViews>
@@ -25,14 +25,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>Sprint</t>
   </si>
   <si>
-    <t>Estado</t>
-  </si>
-  <si>
     <t>Objetivo</t>
   </si>
   <si>
@@ -54,25 +51,10 @@
     <t>Sprint 7</t>
   </si>
   <si>
-    <t>Columna1</t>
-  </si>
-  <si>
-    <t>Columna2</t>
-  </si>
-  <si>
-    <t>Columna3</t>
-  </si>
-  <si>
     <t>Sprint 8</t>
   </si>
   <si>
     <t>Sprint 9</t>
-  </si>
-  <si>
-    <t>Fecha de creacion</t>
-  </si>
-  <si>
-    <t>Conceptos principales</t>
   </si>
   <si>
     <t>Motor</t>
@@ -138,9 +120,6 @@
     <t>DTOs, validaciones, PATCH/PUT, separación de configuración</t>
   </si>
   <si>
-    <t>Persistencia Flash</t>
-  </si>
-  <si>
     <t>Persistencia, serialización, ciclo de vida</t>
   </si>
   <si>
@@ -171,22 +150,37 @@
     <t>Sistema de Configuración</t>
   </si>
   <si>
-    <t>6.1</t>
-  </si>
-  <si>
     <t>Motor configurable</t>
   </si>
   <si>
-    <t>6.2</t>
-  </si>
-  <si>
-    <t>6.3</t>
-  </si>
-  <si>
     <t>Nuevo endpoint PUT /config</t>
   </si>
   <si>
-    <t>GET /config</t>
+    <t>Persistencia de configuración</t>
+  </si>
+  <si>
+    <t>Finalizado</t>
+  </si>
+  <si>
+    <t>Sprint 7.1</t>
+  </si>
+  <si>
+    <t>Sprint 7.2</t>
+  </si>
+  <si>
+    <t>Sprint 6.1</t>
+  </si>
+  <si>
+    <t>Sprint 6.2</t>
+  </si>
+  <si>
+    <t>Crear configurationStorage</t>
+  </si>
+  <si>
+    <t>Objetivo2</t>
+  </si>
+  <si>
+    <t>Implementar persitencia usando Preferences</t>
   </si>
 </sst>
 </file>
@@ -260,7 +254,26 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -284,13 +297,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A61D0C2F-3863-49B5-9DBD-2A45D434E86B}" name="Tabla1" displayName="Tabla1" ref="A2:D17" totalsRowShown="0">
-  <autoFilter ref="A2:D17" xr:uid="{A61D0C2F-3863-49B5-9DBD-2A45D434E86B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A61D0C2F-3863-49B5-9DBD-2A45D434E86B}" name="Tabla1" displayName="Tabla1" ref="A1:D15" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:D15" xr:uid="{A61D0C2F-3863-49B5-9DBD-2A45D434E86B}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{D3E4F5C6-AD58-47DC-B6D4-1B0C795F5FB6}" name="Columna1" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{1A70B391-4605-4E18-BEE1-E86883F9110B}" name="Columna2" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{E01F6D3E-C384-492D-BDC3-F82826119388}" name="Columna3" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{2F2A9E25-6206-42ED-814A-D02DA1BC7341}" name="Fecha de creacion"/>
+    <tableColumn id="1" xr3:uid="{D3E4F5C6-AD58-47DC-B6D4-1B0C795F5FB6}" name="Sprint" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{1A70B391-4605-4E18-BEE1-E86883F9110B}" name="Objetivo" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{E01F6D3E-C384-492D-BDC3-F82826119388}" name="Objetivo2" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{2F2A9E25-6206-42ED-814A-D02DA1BC7341}" name="Finalizado"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -593,7 +606,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AD8F467-8232-41EB-8FA5-FE5849A43A27}">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -609,60 +622,63 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>40</v>
+      </c>
+      <c r="D1" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
-        <v>14</v>
+      <c r="D2" s="4">
+        <v>46224</v>
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>15</v>
+      <c r="A3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>13</v>
       </c>
       <c r="D3" s="4">
         <v>46224</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" ht="30">
       <c r="A4" s="3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D4" s="4">
         <v>46224</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" ht="30">
       <c r="A5" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>18</v>
+        <v>5</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D5" s="4">
         <v>46224</v>
@@ -670,137 +686,119 @@
     </row>
     <row r="6" spans="1:4" ht="30">
       <c r="A6" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>20</v>
+        <v>29</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D6" s="4">
-        <v>46224</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="30">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="45">
       <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>22</v>
+      <c r="B7" t="s">
+        <v>30</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D7" s="4">
-        <v>46224</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="30">
-      <c r="A8" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>25</v>
-      </c>
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="45">
+      <c r="A8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="3"/>
       <c r="D8" s="4">
-        <v>46225</v>
+        <v>46227</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="45">
-      <c r="A9" s="3" t="s">
+      <c r="A9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="4">
+        <v>46228</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="30">
+      <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B9" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="4"/>
-    </row>
-    <row r="10" spans="1:4" ht="45">
-      <c r="A10" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="4"/>
+    </row>
+    <row r="11" spans="1:4" ht="45">
+      <c r="A11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="4"/>
-    </row>
-    <row r="11" spans="1:4" ht="45">
-      <c r="A11" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>42</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="4"/>
     </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="3" t="s">
+    <row r="12" spans="1:4" ht="60">
+      <c r="A12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>43</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="4"/>
     </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="3"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="4"/>
-    </row>
-    <row r="14" spans="1:4" ht="30">
+    <row r="13" spans="1:4" ht="30">
+      <c r="A13" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
       <c r="A14" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" s="4"/>
+        <v>25</v>
+      </c>
     </row>
     <row r="15" spans="1:4" ht="30">
       <c r="A15" s="3" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="30">
-      <c r="A17" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fin sprint 7 y primeras modificaciones sprint 8
</commit_message>
<xml_diff>
--- a/docs/Sprints.xlsx
+++ b/docs/Sprints.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADOS\Documents\CatEater\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FC3ABB8-A4DC-47EB-86CC-0636496B2FF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A29960C6-2C5A-47C1-A122-D5797DBEE8CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="1575" windowWidth="20730" windowHeight="11040" xr2:uid="{B0A1328C-A2DF-43BD-A97C-AEC866E5EF49}"/>
   </bookViews>
@@ -187,7 +187,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -214,6 +214,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -235,7 +243,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -250,11 +258,24 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -274,15 +295,6 @@
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -297,12 +309,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A61D0C2F-3863-49B5-9DBD-2A45D434E86B}" name="Tabla1" displayName="Tabla1" ref="A1:D15" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A61D0C2F-3863-49B5-9DBD-2A45D434E86B}" name="Tabla1" displayName="Tabla1" ref="A1:D15" totalsRowShown="0" headerRowDxfId="3">
   <autoFilter ref="A1:D15" xr:uid="{A61D0C2F-3863-49B5-9DBD-2A45D434E86B}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{D3E4F5C6-AD58-47DC-B6D4-1B0C795F5FB6}" name="Sprint" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{1A70B391-4605-4E18-BEE1-E86883F9110B}" name="Objetivo" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{E01F6D3E-C384-492D-BDC3-F82826119388}" name="Objetivo2" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{D3E4F5C6-AD58-47DC-B6D4-1B0C795F5FB6}" name="Sprint" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{1A70B391-4605-4E18-BEE1-E86883F9110B}" name="Objetivo" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{E01F6D3E-C384-492D-BDC3-F82826119388}" name="Objetivo2" dataDxfId="0"/>
     <tableColumn id="4" xr3:uid="{2F2A9E25-6206-42ED-814A-D02DA1BC7341}" name="Finalizado"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -606,7 +618,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AD8F467-8232-41EB-8FA5-FE5849A43A27}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -614,7 +626,7 @@
     <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -628,7 +640,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -642,7 +654,7 @@
         <v>46224</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
@@ -656,7 +668,7 @@
         <v>46224</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="30">
+    <row r="4" spans="1:6" ht="30">
       <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
@@ -670,7 +682,7 @@
         <v>46224</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="30">
+    <row r="5" spans="1:6" ht="30">
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
@@ -684,7 +696,7 @@
         <v>46224</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="30">
+    <row r="6" spans="1:6" ht="30">
       <c r="A6" s="3" t="s">
         <v>29</v>
       </c>
@@ -698,7 +710,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="45">
+    <row r="7" spans="1:6" ht="45">
       <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
@@ -709,10 +721,10 @@
         <v>20</v>
       </c>
       <c r="D7" s="4">
-        <v>46226</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="45">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="45">
       <c r="A8" t="s">
         <v>37</v>
       </c>
@@ -721,10 +733,10 @@
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="4">
-        <v>46227</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="45">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="45">
       <c r="A9" t="s">
         <v>38</v>
       </c>
@@ -733,10 +745,10 @@
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="4">
-        <v>46228</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="30">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="30">
       <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
@@ -746,9 +758,11 @@
       <c r="C10" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="4"/>
-    </row>
-    <row r="11" spans="1:4" ht="45">
+      <c r="D10" s="4">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="45">
       <c r="A11" t="s">
         <v>35</v>
       </c>
@@ -756,19 +770,24 @@
         <v>39</v>
       </c>
       <c r="C11" s="3"/>
-      <c r="D11" s="4"/>
-    </row>
-    <row r="12" spans="1:4" ht="60">
+      <c r="D11" s="4">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="60">
       <c r="A12" t="s">
         <v>36</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="3"/>
-      <c r="D12" s="4"/>
-    </row>
-    <row r="13" spans="1:4" ht="30">
+      <c r="C12" s="6"/>
+      <c r="D12" s="4">
+        <v>46226</v>
+      </c>
+      <c r="F12" s="7"/>
+    </row>
+    <row r="13" spans="1:6" ht="30">
       <c r="A13" s="3" t="s">
         <v>8</v>
       </c>
@@ -779,7 +798,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:6">
       <c r="A14" s="3" t="s">
         <v>9</v>
       </c>
@@ -790,7 +809,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="30">
+    <row r="15" spans="1:6" ht="30">
       <c r="A15" s="3" t="s">
         <v>26</v>
       </c>

</xml_diff>